<commit_message>
Record audited bug hunt and refresh versioned review artifacts
</commit_message>
<xml_diff>
--- a/docs/audit-workbook.xlsx
+++ b/docs/audit-workbook.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R12f849633f47449b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R53e8be7c4d434471"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policies" sheetId="3" r:id="Re4c2b48b20324499"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly snapshot" sheetId="4" r:id="R54c9a3597135474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort snapshot" sheetId="5" r:id="Rba342da39cfd4470"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loan benchmark" sheetId="6" r:id="Reff58c99b46a48b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Default benchmark" sheetId="7" r:id="R27ea658bd7b4408e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R2993be97a2394fc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R0de4744ae2bf4b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R95bf3c8fe3df45ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R74ab6dd219dd4b4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policies" sheetId="3" r:id="R6051a7224a8f4f10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly snapshot" sheetId="4" r:id="Rcb7902d8c02d443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort snapshot" sheetId="5" r:id="R627ee42f6029443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Loan benchmark" sheetId="6" r:id="R8bd74676443f4f87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Default benchmark" sheetId="7" r:id="Racab1678bd7f43e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="8" r:id="R7e4a7d8205714b1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R1e004d4373fd41cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -543,7 +543,7 @@
         <x:v>Run ID</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>5a88f7bef3fa93d4</x:v>
+        <x:v>438a13c9e03c52a9</x:v>
       </x:c>
       <x:c r="C2" s="2"/>
       <x:c r="D2" s="2"/>
@@ -582,7 +582,7 @@
         <x:v>Model version</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
-        <x:v>0.1.0</x:v>
+        <x:v>0.1.1</x:v>
       </x:c>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="2"/>
@@ -1201,7 +1201,7 @@
         <x:v>Both limits met</x:v>
       </x:c>
       <x:c r="M2" s="2" t="str">
-        <x:v>5a88f7bef3fa93d4</x:v>
+        <x:v>438a13c9e03c52a9</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
@@ -1242,7 +1242,7 @@
         <x:v>Minimum-cash floor breached</x:v>
       </x:c>
       <x:c r="M3" s="2" t="str">
-        <x:v>a2feec5a72facbc3</x:v>
+        <x:v>70d251749e3b54d6</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="20" customHeight="1">
@@ -1283,7 +1283,7 @@
         <x:v>Minimum-cash floor breached</x:v>
       </x:c>
       <x:c r="M4" s="2" t="str">
-        <x:v>5d28e1ac49bb98b2</x:v>
+        <x:v>070bb5007d48fe87</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -50085,7 +50085,7 @@
         <x:v>Simplified equity identity</x:v>
       </x:c>
       <x:c r="B5" s="24" t="n">
-        <x:v>1.45e-27</x:v>
+        <x:v>8e-28</x:v>
       </x:c>
       <x:c r="C5" s="25" t="n">
         <x:v>1e-16</x:v>

</xml_diff>